<commit_message>
added section for committes
</commit_message>
<xml_diff>
--- a/data/cv.xlsx
+++ b/data/cv.xlsx
@@ -1138,6 +1138,16 @@
           <t>college</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2025 - present</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CHS AI Steering Committee, Faculty Member</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>

<commit_message>
Add Mil Med publication and mark Wilson Berry as graduated
Spring 2026 digital measures update: added Bruce Leicht et al. (2025)
"Lower Extremity Symmetry and Normative Values During Functional
Performance Tests in Entry-Level U.S. Marines" to published articles,
and updated Wilson Berry to graduated (MS, Dec 2025).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cv.xlsx
+++ b/data/cv.xlsx
@@ -365,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -1095,6 +1095,39 @@
       <c r="H21" t="inlineStr">
         <is>
           <t>10.1093/milmed/usaf493</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>peer_rev_pub_article</t>
+        </is>
+      </c>
+      <c r="B22" s="2">
+        <v>45983.20833333333</v>
+      </c>
+      <c r="C22">
+        <v>2025</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Bruce Leicht AS, Winters JD, Bergin RT, Carroll B, Djafar T, Green BS, Heebner NR, Fraser JJ, McCloughan NH, Ross J, Sessoms PH, Silder AB, Hoch MC</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Lower Extremity Symmetry and Normative Values During Functional Performance Tests in Entry-Level U.S. Marines</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Mil Med</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>10.1093/milmed/usaf572</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1989,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1964,7 +1997,7 @@
         </is>
       </c>
       <c r="G3">
-        <v>20453</v>
+        <v>20423</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Add MPEES force plate reliability publication and clean up Mil Med entry
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cv.xlsx
+++ b/data/cv.xlsx
@@ -365,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Bruce Leicht AS, Winters JD, Bergin RT, Carroll B, Djafar T, Green BS, Heebner NR, Fraser JJ, McCloughan NH, Ross J, Sessoms PH, Silder AB, Hoch MC</t>
+          <t>Bruce Leicht AS, Winters JD, **Bergin RT**, Carroll B, Djafar T, Green BS, Heebner NR, Fraser JJ, McCloughan NH, Ross J, Sessoms PH, Silder AB, Hoch MC</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1122,12 +1122,50 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Mil Med</t>
+          <t>Military Medicine</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>10.1093/milmed/usaf572</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>peer_rev_pub_article</t>
+        </is>
+      </c>
+      <c r="B23" s="2">
+        <v>46197</v>
+      </c>
+      <c r="C23">
+        <v>2026</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ross JA, **Bergin RT**, Taylor M, Torp DM, Heebner NR, Winters JD, Djafar T, Carroll BA, Hoch MC</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Reliability of Common Force Plate-Based Movement Screens in Males and Females</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Measurement in Physical Education and Exercise Science</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1-8</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>10.1080/1091367X.2026.2692042</t>
         </is>
       </c>
     </row>

</xml_diff>